<commit_message>
More cruft cleanup, finish glen canyon release
</commit_message>
<xml_diff>
--- a/Colorado_River_Math.xlsx
+++ b/Colorado_River_Math.xlsx
@@ -980,7 +980,7 @@
       </c>
       <c r="AJ1" t="inlineStr">
         <is>
-          <t>03/04/2026 04:24PM</t>
+          <t>03/05/2026 05:31AM</t>
         </is>
       </c>
     </row>
@@ -8963,7 +8963,9 @@
       <c r="K28" s="9" t="n">
         <v>9.2049</v>
       </c>
-      <c r="L28" s="10" t="inlineStr"/>
+      <c r="L28" s="10" t="n">
+        <v>7.8931</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="18" t="n">
@@ -9011,7 +9013,9 @@
       <c r="K29" s="9" t="n">
         <v>8.952500000000001</v>
       </c>
-      <c r="L29" s="10" t="inlineStr"/>
+      <c r="L29" s="10" t="n">
+        <v>8.384399999999999</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="18" t="n">
@@ -9059,7 +9063,9 @@
       <c r="K30" s="9" t="n">
         <v>7.8273</v>
       </c>
-      <c r="L30" s="10" t="inlineStr"/>
+      <c r="L30" s="10" t="n">
+        <v>7.9353</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="18" t="n">

</xml_diff>